<commit_message>
Cap nhat hoan thien danh muc hoc vu: Hoc ky, Khoa, Bo mon, Nganh, Lop va Quan ly hoc phan (Phan loai Bo mon & Dung chung)
</commit_message>
<xml_diff>
--- a/sample_imports/05_HocKy_Mau.xlsx
+++ b/sample_imports/05_HocKy_Mau.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
   <si>
     <t>MaHocKy</t>
   </si>
@@ -38,7 +38,7 @@
     <t>HK2223_1</t>
   </si>
   <si>
-    <t>Học kỳ 1 (2022-2023)</t>
+    <t>Học kỳ 1</t>
   </si>
   <si>
     <t>2022-2023</t>
@@ -56,7 +56,7 @@
     <t>HK2223_2</t>
   </si>
   <si>
-    <t>Học kỳ 2 (2022-2023)</t>
+    <t>Học kỳ 2</t>
   </si>
   <si>
     <t>2023-01-16</t>
@@ -68,9 +68,6 @@
     <t>HK2324_1</t>
   </si>
   <si>
-    <t>Học kỳ 1 (2023-2024)</t>
-  </si>
-  <si>
     <t>2023-2024</t>
   </si>
   <si>
@@ -83,9 +80,6 @@
     <t>HK2324_2</t>
   </si>
   <si>
-    <t>Học kỳ 2 (2023-2024)</t>
-  </si>
-  <si>
     <t>2024-01-16</t>
   </si>
   <si>
@@ -95,9 +89,6 @@
     <t>HK2425_1</t>
   </si>
   <si>
-    <t>Học kỳ 1 (2024-2025)</t>
-  </si>
-  <si>
     <t>2024-2025</t>
   </si>
   <si>
@@ -113,9 +104,6 @@
     <t>HK2425_2</t>
   </si>
   <si>
-    <t>Học kỳ 2 (2024-2025)</t>
-  </si>
-  <si>
     <t>2025-01-16</t>
   </si>
   <si>
@@ -126,9 +114,6 @@
   </si>
   <si>
     <t>HK2526_1</t>
-  </si>
-  <si>
-    <t>Học kỳ 1 (2025-2026)</t>
   </si>
   <si>
     <t>2025-2026</t>
@@ -480,12 +465,12 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="10.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="10.569" customWidth="true" style="0"/>
+    <col min="2" max="2" width="24.708" customWidth="true" style="0"/>
+    <col min="3" max="3" width="11.711" customWidth="true" style="0"/>
+    <col min="4" max="4" width="12.854" customWidth="true" style="0"/>
+    <col min="5" max="5" width="13.997" customWidth="true" style="0"/>
+    <col min="6" max="6" width="15.282" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -553,16 +538,16 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>
@@ -570,19 +555,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E5" t="s">
         <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
       </c>
       <c r="F5" t="s">
         <v>11</v>
@@ -590,62 +575,62 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
         <v>31</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: cap nhat database quanly_doan, giao dien sinh vien, bo loc he thong va xoa key .env
</commit_message>
<xml_diff>
--- a/sample_imports/05_HocKy_Mau.xlsx
+++ b/sample_imports/05_HocKy_Mau.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
   <si>
     <t>MaHocKy</t>
   </si>
@@ -38,7 +38,7 @@
     <t>HK2223_1</t>
   </si>
   <si>
-    <t>Học kỳ 1</t>
+    <t>Học kỳ 1 (2022-2023)</t>
   </si>
   <si>
     <t>2022-2023</t>
@@ -56,7 +56,7 @@
     <t>HK2223_2</t>
   </si>
   <si>
-    <t>Học kỳ 2</t>
+    <t>Học kỳ 2 (2022-2023)</t>
   </si>
   <si>
     <t>2023-01-16</t>
@@ -68,6 +68,9 @@
     <t>HK2324_1</t>
   </si>
   <si>
+    <t>Học kỳ 1 (2023-2024)</t>
+  </si>
+  <si>
     <t>2023-2024</t>
   </si>
   <si>
@@ -80,6 +83,9 @@
     <t>HK2324_2</t>
   </si>
   <si>
+    <t>Học kỳ 2 (2023-2024)</t>
+  </si>
+  <si>
     <t>2024-01-16</t>
   </si>
   <si>
@@ -89,6 +95,9 @@
     <t>HK2425_1</t>
   </si>
   <si>
+    <t>Học kỳ 1 (2024-2025)</t>
+  </si>
+  <si>
     <t>2024-2025</t>
   </si>
   <si>
@@ -104,6 +113,9 @@
     <t>HK2425_2</t>
   </si>
   <si>
+    <t>Học kỳ 2 (2024-2025)</t>
+  </si>
+  <si>
     <t>2025-01-16</t>
   </si>
   <si>
@@ -114,6 +126,9 @@
   </si>
   <si>
     <t>HK2526_1</t>
+  </si>
+  <si>
+    <t>Học kỳ 1 (2025-2026)</t>
   </si>
   <si>
     <t>2025-2026</t>
@@ -465,12 +480,12 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="10.569" customWidth="true" style="0"/>
-    <col min="2" max="2" width="24.708" customWidth="true" style="0"/>
-    <col min="3" max="3" width="11.711" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" customWidth="true" style="0"/>
-    <col min="5" max="5" width="13.997" customWidth="true" style="0"/>
-    <col min="6" max="6" width="15.282" customWidth="true" style="0"/>
+    <col min="1" max="1" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="24.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="15.282" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -538,16 +553,16 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>
@@ -555,19 +570,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
         <v>11</v>
@@ -575,62 +590,62 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" t="s">
         <v>35</v>
-      </c>
-      <c r="F8" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: cap nhat quy trinh khoa luan 5 cap, xem nhanh de cuong PDF.js, xuat sample imports excel va README chuan
</commit_message>
<xml_diff>
--- a/sample_imports/05_HocKy_Mau.xlsx
+++ b/sample_imports/05_HocKy_Mau.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="05_HocKy_Mau" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
   <si>
     <t>MaHocKy</t>
   </si>
@@ -35,109 +35,70 @@
     <t>TrangThai</t>
   </si>
   <si>
-    <t>HK2223_1</t>
-  </si>
-  <si>
-    <t>Học kỳ 1 (2022-2023)</t>
-  </si>
-  <si>
-    <t>2022-2023</t>
-  </si>
-  <si>
-    <t>2022-09-05</t>
-  </si>
-  <si>
-    <t>2023-01-15</t>
+    <t>HK2627_1</t>
+  </si>
+  <si>
+    <t>Học kỳ 1</t>
+  </si>
+  <si>
+    <t>2026-2027</t>
+  </si>
+  <si>
+    <t>2026-02-01</t>
+  </si>
+  <si>
+    <t>2026-12-31</t>
+  </si>
+  <si>
+    <t>Đang diễn ra</t>
+  </si>
+  <si>
+    <t>HK2526_1</t>
+  </si>
+  <si>
+    <t>Học kỳ 1 (2025-2026)</t>
+  </si>
+  <si>
+    <t>2025-2026</t>
+  </si>
+  <si>
+    <t>2025-09-01</t>
+  </si>
+  <si>
+    <t>2026-01-15</t>
+  </si>
+  <si>
+    <t>Chưa bắt đầu</t>
+  </si>
+  <si>
+    <t>HK2425_2</t>
+  </si>
+  <si>
+    <t>Học kỳ 2 (2024-2025)</t>
+  </si>
+  <si>
+    <t>2024-2025</t>
+  </si>
+  <si>
+    <t>2025-02-15</t>
+  </si>
+  <si>
+    <t>2025-06-30</t>
   </si>
   <si>
     <t>Đã kết thúc</t>
   </si>
   <si>
-    <t>HK2223_2</t>
-  </si>
-  <si>
-    <t>Học kỳ 2 (2022-2023)</t>
-  </si>
-  <si>
-    <t>2023-01-16</t>
-  </si>
-  <si>
-    <t>2023-06-10</t>
-  </si>
-  <si>
-    <t>HK2324_1</t>
-  </si>
-  <si>
-    <t>Học kỳ 1 (2023-2024)</t>
-  </si>
-  <si>
-    <t>2023-2024</t>
-  </si>
-  <si>
-    <t>2023-09-05</t>
-  </si>
-  <si>
-    <t>2024-01-15</t>
-  </si>
-  <si>
-    <t>HK2324_2</t>
-  </si>
-  <si>
-    <t>Học kỳ 2 (2023-2024)</t>
-  </si>
-  <si>
-    <t>2024-01-16</t>
-  </si>
-  <si>
-    <t>2024-06-10</t>
-  </si>
-  <si>
     <t>HK2425_1</t>
   </si>
   <si>
     <t>Học kỳ 1 (2024-2025)</t>
   </si>
   <si>
-    <t>2024-2025</t>
-  </si>
-  <si>
-    <t>2024-09-05</t>
+    <t>2024-09-01</t>
   </si>
   <si>
     <t>2025-01-15</t>
-  </si>
-  <si>
-    <t>Đang diễn ra</t>
-  </si>
-  <si>
-    <t>HK2425_2</t>
-  </si>
-  <si>
-    <t>Học kỳ 2 (2024-2025)</t>
-  </si>
-  <si>
-    <t>2025-01-16</t>
-  </si>
-  <si>
-    <t>2025-06-10</t>
-  </si>
-  <si>
-    <t>Chưa bắt đầu</t>
-  </si>
-  <si>
-    <t>HK2526_1</t>
-  </si>
-  <si>
-    <t>Học kỳ 1 (2025-2026)</t>
-  </si>
-  <si>
-    <t>2025-2026</t>
-  </si>
-  <si>
-    <t>2025-09-05</t>
-  </si>
-  <si>
-    <t>2026-01-15</t>
   </si>
 </sst>
 </file>
@@ -145,7 +106,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -155,16 +116,31 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00529B"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -172,12 +148,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,175 +489,115 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="11.569" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="24.708" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="16.282" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="15.282" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" customHeight="1" ht="28">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F3" t="s">
-        <v>11</v>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
+      <c r="C4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F4" t="s">
-        <v>11</v>
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="A5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>